<commit_message>
Use a neutral persona example (data analysts and ops) throughout
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FyCN5j8pg1ztCe2QPjBLX5
</commit_message>
<xml_diff>
--- a/sheet/valari-template.xlsx
+++ b/sheet/valari-template.xlsx
@@ -758,7 +758,7 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Senior UX Researcher</t>
+          <t>Senior Data Analyst</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>Example row. Ran the research repository rollout to 3 teams.</t>
+          <t>Example row. Ran the analytics rollout to 3 teams.</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Director of Design</t>
+          <t>Director of Operations</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs(examples): generalize persona examples to analytics roles
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FyCN5j8pg1ztCe2QPjBLX5
</commit_message>
<xml_diff>
--- a/sheet/valari-template.xlsx
+++ b/sheet/valari-template.xlsx
@@ -758,7 +758,7 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Senior UX Researcher</t>
+          <t>Senior Data Analyst</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>Example row. Ran the research repository rollout to 3 teams.</t>
+          <t>Example row. Ran the analytics rollout to 3 teams.</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Director of Design</t>
+          <t>Director of Operations</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">

</xml_diff>

<commit_message>
revert: restore original persona examples
This reverts commit 69e513bac36ef8cacb28ad293b3304e75c319559.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FyCN5j8pg1ztCe2QPjBLX5
</commit_message>
<xml_diff>
--- a/sheet/valari-template.xlsx
+++ b/sheet/valari-template.xlsx
@@ -758,7 +758,7 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Senior Data Analyst</t>
+          <t>Senior UX Researcher</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>Example row. Ran the analytics rollout to 3 teams.</t>
+          <t>Example row. Ran the research repository rollout to 3 teams.</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Director of Operations</t>
+          <t>Director of Design</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Restore the UX researcher and designer persona example
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FyCN5j8pg1ztCe2QPjBLX5
</commit_message>
<xml_diff>
--- a/sheet/valari-template.xlsx
+++ b/sheet/valari-template.xlsx
@@ -758,7 +758,7 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Senior Data Analyst</t>
+          <t>Senior UX Researcher</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>Example row. Ran the analytics rollout to 3 teams.</t>
+          <t>Example row. Ran the research repository rollout to 3 teams.</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Director of Operations</t>
+          <t>Director of Design</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">

</xml_diff>